<commit_message>
Validación Grupo Pérez: Grupo Pérez arriba, 4 empresas (Basarili, Agro, Superior, MGP) con conteo en vivo, consulta de vendedores sin clave (4 letras), cargar archivo por empresa, Integra Supply con clave
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Plantilla clientes Grupo Perez.xlsx
+++ b/Plantilla clientes Grupo Perez.xlsx
@@ -613,7 +613,7 @@
       <formula1>"Negocio,Persona natural"</formula1>
     </dataValidation>
     <dataValidation sqref="K2:K2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"FEROZ,ALPACA,FORTIA,INTEGRA SUPPLY"</formula1>
+      <formula1>"BASARILI,AGRO,SUPERIOR,MGP"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -635,12 +635,9 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Plantilla de clientes · Grupo Pérez (Feroz · Alpaca · Fortia · Integra Supply)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
+          <t>Plantilla de clientes · Grupo Pérez (Basarili · Agro · Superior · MGP)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -673,7 +670,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>5. EMPRESA: FEROZ, ALPACA, FORTIA o INTEGRA SUPPLY. Si la dejas vacía, queda la empresa de la clave con que subes el archivo.</t>
+          <t>5. EMPRESA: BASARILI, AGRO, SUPERIOR o MGP. Es solo informativa: al subir el archivo, la empresa que eliges en la página es la que queda.</t>
         </is>
       </c>
     </row>
@@ -687,7 +684,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>7. Sube el archivo en ferozsafetywear.com/validar.html → pestaña Vendedores → Subir el Excel.</t>
+          <t>7. Sube el archivo en ferozsafetywear.com/validar.html → elige tu empresa, escribe su clave y usa "Cargar archivo".</t>
         </is>
       </c>
     </row>

</xml_diff>